<commit_message>
DATA-04: rebrand synthetic sources and prepare Valentino product data
</commit_message>
<xml_diff>
--- a/generated/sources/internal_comms/voice_of_customer/instore_feedback_survey_export_20261022.xlsx
+++ b/generated/sources/internal_comms/voice_of_customer/instore_feedback_survey_export_20261022.xlsx
@@ -807,7 +807,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Ambrine marrone 1</t>
+          <t>Amalia marrone 1</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>polo navy L</t>
+          <t>jersey polo navy L</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Maire black</t>
+          <t>Aurea black</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Maire noire</t>
+          <t>Aurea noire</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Maire black 1</t>
+          <t>Aurea black 1</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>POLARIS太好看了！</t>
+          <t>ASTRA太好看了！</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Le Polaris taille vraiment petit, et à ce prix…</t>
+          <t>Le Astra taille vraiment petit, et à ce prix…</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Polaris Jacke viel zu klein geschnitten für den Preis</t>
+          <t>Astra Jacke viel zu klein geschnitten für den Preis</t>
         </is>
       </c>
     </row>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>POLARIS CAPE 白色 L</t>
+          <t>ASTRA CAPE 白色 L</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Maire black 0</t>
+          <t>Aurea black 0</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>maire black</t>
+          <t>aurea black</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Maire black</t>
+          <t>Aurea black</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Ilvaro pink</t>
+          <t>Iridia pink</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>粉色ILVARO</t>
+          <t>粉色IRIDIA</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>ILVARO 粉色</t>
+          <t>IRIDIA 粉色</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Ilvaro 粉紅色</t>
+          <t>Iridia 粉紅色</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>ILVARO ピンク</t>
+          <t>IRIDIA ピンク</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Maya negra 4</t>
+          <t>Nova negra 4</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>MAIRE 黑色</t>
+          <t>AUREA 黑色</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -2639,7 +2639,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>ILVARO 粉色 0</t>
+          <t>IRIDIA 粉色 0</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Ilvaro pink 0</t>
+          <t>Iridia pink 0</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Maya negra</t>
+          <t>Nova negra</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3113,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>TIB拉链质量太差</t>
+          <t>VEL拉链质量太差</t>
         </is>
       </c>
     </row>
@@ -3209,7 +3209,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>black Maire size 1</t>
+          <t>black Aurea size 1</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -3417,7 +3417,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>ARNEBが大きめでした。店員さんのアドバイスで小さいサイズに</t>
+          <t>ARTEMが大きめでした。店員さんのアドバイスで小さいサイズに</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Gilet TIB fermeture cassée après 3 semaines. Déçue.</t>
+          <t>Gilet VEL fermeture cassée après 3 semaines. Déçue.</t>
         </is>
       </c>
     </row>
@@ -3564,7 +3564,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Ambrine brown</t>
+          <t>Amalia brown</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -3618,7 +3618,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Logo cardigan M</t>
+          <t>Vlogo Cardigan M</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -4186,7 +4186,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>MAIRE ブラック 2</t>
+          <t>AUREA ブラック 2</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -4243,7 +4243,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>La Maya negra por fin. Muy amables</t>
+          <t>La Nova negra por fin. Muy amables</t>
         </is>
       </c>
     </row>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>TIB gilet zip broke within a month. Exchanged, but not great.</t>
+          <t>VEL gilet zip broke within a month. Exchanged, but not great.</t>
         </is>
       </c>
     </row>
@@ -4486,7 +4486,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Maya schwarz 3</t>
+          <t>Nova schwarz 3</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -4543,7 +4543,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>Finally a proper down jacket weather in Milan! Maya fits perfectly</t>
+          <t>Finally a proper down jacket weather in Milan! Nova fits perfectly</t>
         </is>
       </c>
     </row>
@@ -4592,7 +4592,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>Ilvaro black 0</t>
+          <t>Iridia black 0</t>
         </is>
       </c>
     </row>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>Freezing outside, great to find my size of Karakorum</t>
+          <t>Freezing outside, great to find my size of Cosimo</t>
         </is>
       </c>
     </row>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Maire black 0</t>
+          <t>Aurea black 0</t>
         </is>
       </c>
     </row>
@@ -5118,7 +5118,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>Maire black</t>
+          <t>Aurea black</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>Ambrine marron 1</t>
+          <t>Amalia marron 1</t>
         </is>
       </c>
       <c r="M94" t="inlineStr">
@@ -5472,7 +5472,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>Presa finalmente la Maire nera!! 🖤</t>
+          <t>Presa finalmente la Aurea nera!! 🖤</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DATA-04: Valentino rebrand and visual product data (#158)
* DATA-04: start

* DATA-04: rebrand synthetic sources and prepare Valentino product data

* DATA-04: refresh rebranded replay inputs and insight hashes
</commit_message>
<xml_diff>
--- a/generated/sources/internal_comms/voice_of_customer/instore_feedback_survey_export_20261022.xlsx
+++ b/generated/sources/internal_comms/voice_of_customer/instore_feedback_survey_export_20261022.xlsx
@@ -807,7 +807,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Ambrine marrone 1</t>
+          <t>Amalia marrone 1</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>polo navy L</t>
+          <t>jersey polo navy L</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Maire black</t>
+          <t>Aurea black</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Maire noire</t>
+          <t>Aurea noire</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Maire black 1</t>
+          <t>Aurea black 1</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>POLARIS太好看了！</t>
+          <t>ASTRA太好看了！</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Le Polaris taille vraiment petit, et à ce prix…</t>
+          <t>Le Astra taille vraiment petit, et à ce prix…</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Polaris Jacke viel zu klein geschnitten für den Preis</t>
+          <t>Astra Jacke viel zu klein geschnitten für den Preis</t>
         </is>
       </c>
     </row>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>POLARIS CAPE 白色 L</t>
+          <t>ASTRA CAPE 白色 L</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Maire black 0</t>
+          <t>Aurea black 0</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>maire black</t>
+          <t>aurea black</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Maire black</t>
+          <t>Aurea black</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Ilvaro pink</t>
+          <t>Iridia pink</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>粉色ILVARO</t>
+          <t>粉色IRIDIA</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>ILVARO 粉色</t>
+          <t>IRIDIA 粉色</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Ilvaro 粉紅色</t>
+          <t>Iridia 粉紅色</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>ILVARO ピンク</t>
+          <t>IRIDIA ピンク</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Maya negra 4</t>
+          <t>Nova negra 4</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>MAIRE 黑色</t>
+          <t>AUREA 黑色</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -2639,7 +2639,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>ILVARO 粉色 0</t>
+          <t>IRIDIA 粉色 0</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Ilvaro pink 0</t>
+          <t>Iridia pink 0</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Maya negra</t>
+          <t>Nova negra</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3113,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>TIB拉链质量太差</t>
+          <t>VEL拉链质量太差</t>
         </is>
       </c>
     </row>
@@ -3209,7 +3209,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>black Maire size 1</t>
+          <t>black Aurea size 1</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -3417,7 +3417,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>ARNEBが大きめでした。店員さんのアドバイスで小さいサイズに</t>
+          <t>ARTEMが大きめでした。店員さんのアドバイスで小さいサイズに</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Gilet TIB fermeture cassée après 3 semaines. Déçue.</t>
+          <t>Gilet VEL fermeture cassée après 3 semaines. Déçue.</t>
         </is>
       </c>
     </row>
@@ -3564,7 +3564,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Ambrine brown</t>
+          <t>Amalia brown</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -3618,7 +3618,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Logo cardigan M</t>
+          <t>Vlogo Cardigan M</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -4186,7 +4186,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>MAIRE ブラック 2</t>
+          <t>AUREA ブラック 2</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -4243,7 +4243,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>La Maya negra por fin. Muy amables</t>
+          <t>La Nova negra por fin. Muy amables</t>
         </is>
       </c>
     </row>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>TIB gilet zip broke within a month. Exchanged, but not great.</t>
+          <t>VEL gilet zip broke within a month. Exchanged, but not great.</t>
         </is>
       </c>
     </row>
@@ -4486,7 +4486,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Maya schwarz 3</t>
+          <t>Nova schwarz 3</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -4543,7 +4543,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>Finally a proper down jacket weather in Milan! Maya fits perfectly</t>
+          <t>Finally a proper down jacket weather in Milan! Nova fits perfectly</t>
         </is>
       </c>
     </row>
@@ -4592,7 +4592,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>Ilvaro black 0</t>
+          <t>Iridia black 0</t>
         </is>
       </c>
     </row>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>Freezing outside, great to find my size of Karakorum</t>
+          <t>Freezing outside, great to find my size of Cosimo</t>
         </is>
       </c>
     </row>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Maire black 0</t>
+          <t>Aurea black 0</t>
         </is>
       </c>
     </row>
@@ -5118,7 +5118,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>Maire black</t>
+          <t>Aurea black</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>Ambrine marron 1</t>
+          <t>Amalia marron 1</t>
         </is>
       </c>
       <c r="M94" t="inlineStr">
@@ -5472,7 +5472,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>Presa finalmente la Maire nera!! 🖤</t>
+          <t>Presa finalmente la Aurea nera!! 🖤</t>
         </is>
       </c>
     </row>

</xml_diff>